<commit_message>
fix: scripts should include autofit for columns
</commit_message>
<xml_diff>
--- a/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
+++ b/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
@@ -586,28 +586,28 @@
   <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="16" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="9" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
fix: added a shared module implementing one consistent coloring rule
</commit_message>
<xml_diff>
--- a/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
+++ b/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,8 +29,14 @@
       <b val="1"/>
     </font>
     <font/>
+    <font>
+      <color rgb="00006100"/>
+    </font>
+    <font>
+      <color rgb="009C6500"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -51,20 +57,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8CBAD"/>
-        <bgColor rgb="00F8CBAD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
         <bgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BDD7EE"/>
-        <bgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -185,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -196,26 +190,20 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1108,7 +1096,7 @@
       <c r="Q7" s="5" t="n">
         <v>0.9691773328957446</v>
       </c>
-      <c r="R7" s="10" t="inlineStr">
+      <c r="R7" s="6" t="inlineStr">
         <is>
           <t>Qwen 7B</t>
         </is>
@@ -1122,7 +1110,7 @@
       <c r="U7" s="5" t="n">
         <v>0.9121212121212121</v>
       </c>
-      <c r="V7" s="11" t="inlineStr">
+      <c r="V7" s="10" t="inlineStr">
         <is>
           <t>tie</t>
         </is>
@@ -1200,7 +1188,7 @@
       <c r="U8" s="8" t="n">
         <v>0.9215686274509802</v>
       </c>
-      <c r="V8" s="12" t="inlineStr">
+      <c r="V8" s="11" t="inlineStr">
         <is>
           <t>tie</t>
         </is>
@@ -1268,7 +1256,7 @@
       <c r="Q9" s="5" t="n">
         <v>0.9465645331784954</v>
       </c>
-      <c r="R9" s="11" t="inlineStr">
+      <c r="R9" s="10" t="inlineStr">
         <is>
           <t>tie</t>
         </is>
@@ -1282,7 +1270,7 @@
       <c r="U9" s="5" t="n">
         <v>0.8803827751196173</v>
       </c>
-      <c r="V9" s="11" t="inlineStr">
+      <c r="V9" s="10" t="inlineStr">
         <is>
           <t>tie</t>
         </is>
@@ -1360,7 +1348,7 @@
       <c r="U10" s="5" t="n">
         <v>0.8451957295373673</v>
       </c>
-      <c r="V10" s="13" t="inlineStr">
+      <c r="V10" s="6" t="inlineStr">
         <is>
           <t>Qwen 3B</t>
         </is>

</xml_diff>

<commit_message>
fix: a tie includes not only exact equality, but also any spread within 1% of the larger value
</commit_message>
<xml_diff>
--- a/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
+++ b/experiments/01_term_expansion_by_model/report/dev_v1_cleaned_model_comparison.xlsx
@@ -591,7 +591,7 @@
     <col width="20" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
     <col width="20" customWidth="1" min="19" max="19"/>
     <col width="20" customWidth="1" min="20" max="20"/>
     <col width="20" customWidth="1" min="21" max="21"/>
@@ -1018,9 +1018,9 @@
       <c r="Q6" s="5" t="n">
         <v>0.974571620813397</v>
       </c>
-      <c r="R6" s="6" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="R6" s="10" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
       <c r="S6" s="5" t="n">
@@ -1032,9 +1032,9 @@
       <c r="U6" s="5" t="n">
         <v>0.9400921658986178</v>
       </c>
-      <c r="V6" s="6" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="V6" s="10" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
     </row>
@@ -1096,9 +1096,9 @@
       <c r="Q7" s="5" t="n">
         <v>0.9691773328957446</v>
       </c>
-      <c r="R7" s="6" t="inlineStr">
-        <is>
-          <t>Qwen 7B</t>
+      <c r="R7" s="10" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
       <c r="S7" s="5" t="n">
@@ -1174,9 +1174,9 @@
       <c r="Q8" s="8" t="n">
         <v>0.9720018885741264</v>
       </c>
-      <c r="R8" s="9" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="R8" s="11" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
       <c r="S8" s="8" t="n">
@@ -1334,9 +1334,9 @@
       <c r="Q10" s="5" t="n">
         <v>0.9256646630747351</v>
       </c>
-      <c r="R10" s="6" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="R10" s="10" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
       <c r="S10" s="5" t="n">
@@ -1412,9 +1412,9 @@
       <c r="Q11" s="8" t="n">
         <v>0.9585570898862037</v>
       </c>
-      <c r="R11" s="9" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="R11" s="11" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
       <c r="S11" s="8" t="n">
@@ -1426,9 +1426,9 @@
       <c r="U11" s="8" t="n">
         <v>0.9109090909090911</v>
       </c>
-      <c r="V11" s="9" t="inlineStr">
-        <is>
-          <t>GPT</t>
+      <c r="V11" s="11" t="inlineStr">
+        <is>
+          <t>tie</t>
         </is>
       </c>
     </row>

</xml_diff>